<commit_message>
Update trading calendar and daily records
</commit_message>
<xml_diff>
--- a/monitor_xlsx/20260120.xlsx
+++ b/monitor_xlsx/20260120.xlsx
@@ -999,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2297,6 +2297,59 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3030</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>德律</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>175</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2853</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>-1225</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-2318</v>
+      </c>
+      <c r="H23" t="n">
+        <v>153</v>
+      </c>
+      <c r="I23" t="n">
+        <v>305</v>
+      </c>
+      <c r="J23" t="n">
+        <v>84</v>
+      </c>
+      <c r="K23" t="n">
+        <v>6885</v>
+      </c>
+      <c r="L23" t="n">
+        <v>34799</v>
+      </c>
+      <c r="M23" t="n">
+        <v>-58815</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>偏空</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>

</xml_diff>